<commit_message>
Add dictionary conditional formatting & build sheets from csv
csv is wip and currently errors if issues are printed
</commit_message>
<xml_diff>
--- a/tests/test-files/data-issues.xlsx
+++ b/tests/test-files/data-issues.xlsx
@@ -8,16 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{677E77E8-DDDC-4AC9-BB5E-E9D6F60EBD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D701B2C-02FF-4020-9E32-9243051A9ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Data Dictionary" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Issues" sheetId="6" state="visible" r:id="rId4"/>
+    <sheet name="ref" sheetId="7" state="hidden" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="valid_groups">'ref'!$A$2:$A$5</definedName>
+  </definedNames>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="472">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="471">
   <si>
     <t>year</t>
   </si>
@@ -2533,9 +2537,6 @@
     <t>a</t>
   </si>
   <si>
-    <t>d</t>
-  </si>
-  <si>
     <t>f</t>
   </si>
 </sst>
@@ -2671,7 +2672,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2713,9 +2714,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0">
@@ -3495,8 +3493,8 @@
       <c r="J2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>469</v>
+      <c r="K2" s="1">
+        <v>29</v>
       </c>
       <c r="L2" s="1">
         <v>36</v>
@@ -3617,8 +3615,8 @@
       <c r="J3" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>469</v>
+      <c r="K3" s="1">
+        <v>34</v>
       </c>
       <c r="L3" s="1">
         <v>46</v>
@@ -3739,8 +3737,8 @@
       <c r="J4" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>469</v>
+      <c r="K4" s="1">
+        <v>20</v>
       </c>
       <c r="L4" s="1">
         <v>70</v>
@@ -3861,8 +3859,8 @@
       <c r="J5" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>469</v>
+      <c r="K5" s="1">
+        <v>18</v>
       </c>
       <c r="L5" s="1">
         <v>70</v>
@@ -3983,8 +3981,8 @@
       <c r="J6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>469</v>
+      <c r="K6" s="1">
+        <v>28</v>
       </c>
       <c r="L6" s="1">
         <v>43</v>
@@ -3992,8 +3990,8 @@
       <c r="M6" s="1">
         <v>29</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>470</v>
+      <c r="N6" s="1">
+        <v>1.03</v>
       </c>
       <c r="O6" s="1">
         <v>95.8</v>
@@ -4105,8 +4103,8 @@
       <c r="J7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K7" s="1" t="s">
-        <v>469</v>
+      <c r="K7" s="1">
+        <v>33</v>
       </c>
       <c r="L7" s="1">
         <v>54</v>
@@ -4123,8 +4121,8 @@
       <c r="P7" s="1">
         <v>2.02</v>
       </c>
-      <c r="Q7" s="1" t="s">
-        <v>471</v>
+      <c r="Q7" s="1">
+        <v>1.6</v>
       </c>
       <c r="R7" s="1">
         <v>27.7</v>
@@ -4227,8 +4225,8 @@
       <c r="J8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K8" s="1" t="s">
-        <v>469</v>
+      <c r="K8" s="1">
+        <v>76</v>
       </c>
       <c r="L8" s="1">
         <v>21</v>
@@ -4349,8 +4347,8 @@
       <c r="J9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K9" s="1" t="s">
-        <v>469</v>
+      <c r="K9" s="1">
+        <v>71</v>
       </c>
       <c r="L9" s="1">
         <v>27</v>
@@ -4474,8 +4472,8 @@
       <c r="J10" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K10" s="1" t="s">
-        <v>469</v>
+      <c r="K10" s="1">
+        <v>55</v>
       </c>
       <c r="L10" s="1">
         <v>37</v>
@@ -4596,8 +4594,8 @@
       <c r="J11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K11" s="1" t="s">
-        <v>469</v>
+      <c r="K11" s="1">
+        <v>53</v>
       </c>
       <c r="L11" s="1">
         <v>41</v>
@@ -4605,8 +4603,8 @@
       <c r="M11" s="1">
         <v>6</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>470</v>
+      <c r="N11" s="1">
+        <v>1.1599999999999999</v>
       </c>
       <c r="O11" s="1">
         <v>58.5</v>
@@ -4718,8 +4716,8 @@
       <c r="J12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K12" s="1" t="s">
-        <v>469</v>
+      <c r="K12" s="1">
+        <v>42</v>
       </c>
       <c r="L12" s="1">
         <v>34</v>
@@ -4840,8 +4838,8 @@
       <c r="J13" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K13" s="1" t="s">
-        <v>469</v>
+      <c r="K13" s="1">
+        <v>75</v>
       </c>
       <c r="L13" s="1">
         <v>23</v>
@@ -4962,8 +4960,8 @@
       <c r="J14" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>469</v>
+      <c r="K14" s="1">
+        <v>74</v>
       </c>
       <c r="L14" s="1">
         <v>20</v>
@@ -5081,8 +5079,8 @@
       <c r="J15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>469</v>
+      <c r="K15" s="1">
+        <v>61</v>
       </c>
       <c r="L15" s="1">
         <v>33</v>
@@ -5099,8 +5097,8 @@
       <c r="P15" s="1">
         <v>1.33</v>
       </c>
-      <c r="Q15" s="1" t="s">
-        <v>470</v>
+      <c r="Q15" s="1">
+        <v>20.6</v>
       </c>
       <c r="R15" s="1">
         <v>126.8</v>
@@ -5203,8 +5201,8 @@
       <c r="J16" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K16" s="1" t="s">
-        <v>469</v>
+      <c r="K16" s="1">
+        <v>43</v>
       </c>
       <c r="L16" s="1">
         <v>46</v>
@@ -5325,8 +5323,8 @@
       <c r="J17" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K17" s="1" t="s">
-        <v>469</v>
+      <c r="K17" s="1">
+        <v>49</v>
       </c>
       <c r="L17" s="1">
         <v>39</v>
@@ -5444,8 +5442,8 @@
       <c r="J18" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K18" s="1" t="s">
-        <v>469</v>
+      <c r="K18" s="1">
+        <v>44</v>
       </c>
       <c r="L18" s="1">
         <v>39</v>
@@ -5453,8 +5451,8 @@
       <c r="M18" s="1">
         <v>17</v>
       </c>
-      <c r="N18" s="1" t="s">
-        <v>469</v>
+      <c r="N18" s="1">
+        <v>1.4</v>
       </c>
       <c r="O18" s="1">
         <v>90.9</v>
@@ -5563,8 +5561,8 @@
       <c r="J19" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>469</v>
+      <c r="K19" s="1">
+        <v>19</v>
       </c>
       <c r="L19" s="1">
         <v>53</v>
@@ -5685,8 +5683,8 @@
       <c r="J20" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K20" s="1" t="s">
-        <v>469</v>
+      <c r="K20" s="1">
+        <v>18</v>
       </c>
       <c r="L20" s="1">
         <v>66</v>
@@ -5807,8 +5805,8 @@
       <c r="J21" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>469</v>
+      <c r="K21" s="1">
+        <v>42</v>
       </c>
       <c r="L21" s="1">
         <v>48</v>
@@ -5929,8 +5927,8 @@
       <c r="J22" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K22" s="1" t="s">
-        <v>469</v>
+      <c r="K22" s="1">
+        <v>27</v>
       </c>
       <c r="L22" s="1">
         <v>59</v>
@@ -6051,8 +6049,8 @@
       <c r="J23" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>469</v>
+      <c r="K23" s="1">
+        <v>68</v>
       </c>
       <c r="L23" s="1">
         <v>28</v>
@@ -6173,8 +6171,8 @@
       <c r="J24" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>469</v>
+      <c r="K24" s="1">
+        <v>44</v>
       </c>
       <c r="L24" s="1">
         <v>42</v>
@@ -6295,8 +6293,8 @@
       <c r="J25" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>469</v>
+      <c r="K25" s="1">
+        <v>55</v>
       </c>
       <c r="L25" s="1">
         <v>39</v>
@@ -6420,8 +6418,8 @@
       <c r="J26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K26" s="1" t="s">
-        <v>469</v>
+      <c r="K26" s="1">
+        <v>18</v>
       </c>
       <c r="L26" s="1">
         <v>73</v>
@@ -6542,8 +6540,8 @@
       <c r="J27" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K27" s="1" t="s">
-        <v>469</v>
+      <c r="K27" s="1">
+        <v>63</v>
       </c>
       <c r="L27" s="1">
         <v>31</v>
@@ -6664,8 +6662,8 @@
       <c r="J28" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K28" s="1" t="s">
-        <v>469</v>
+      <c r="K28" s="1">
+        <v>67</v>
       </c>
       <c r="L28" s="1">
         <v>26</v>
@@ -6786,8 +6784,8 @@
       <c r="J29" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K29" s="1" t="s">
-        <v>469</v>
+      <c r="K29" s="1">
+        <v>36</v>
       </c>
       <c r="L29" s="1">
         <v>54</v>
@@ -6908,8 +6906,8 @@
       <c r="J30" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K30" s="1" t="s">
-        <v>469</v>
+      <c r="K30" s="1">
+        <v>31</v>
       </c>
       <c r="L30" s="1">
         <v>50</v>
@@ -7033,8 +7031,8 @@
       <c r="J31" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K31" s="1" t="s">
-        <v>469</v>
+      <c r="K31" s="1">
+        <v>37</v>
       </c>
       <c r="L31" s="1">
         <v>51</v>
@@ -7155,8 +7153,8 @@
       <c r="J32" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K32" s="1" t="s">
-        <v>469</v>
+      <c r="K32" s="1">
+        <v>39</v>
       </c>
       <c r="L32" s="1">
         <v>43</v>
@@ -7280,8 +7278,8 @@
       <c r="J33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K33" s="1" t="s">
-        <v>469</v>
+      <c r="K33" s="1">
+        <v>19</v>
       </c>
       <c r="L33" s="1">
         <v>60</v>
@@ -7402,8 +7400,8 @@
       <c r="J34" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K34" s="1" t="s">
-        <v>469</v>
+      <c r="K34" s="1">
+        <v>16</v>
       </c>
       <c r="L34" s="1">
         <v>62</v>
@@ -7524,8 +7522,8 @@
       <c r="J35" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K35" s="1" t="s">
-        <v>469</v>
+      <c r="K35" s="1">
+        <v>17</v>
       </c>
       <c r="L35" s="1">
         <v>61</v>
@@ -7646,8 +7644,8 @@
       <c r="J36" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K36" s="1" t="s">
-        <v>469</v>
+      <c r="K36" s="1">
+        <v>22</v>
       </c>
       <c r="L36" s="1">
         <v>57</v>
@@ -7768,8 +7766,8 @@
       <c r="J37" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K37" s="1" t="s">
-        <v>469</v>
+      <c r="K37" s="1">
+        <v>43</v>
       </c>
       <c r="L37" s="1">
         <v>42</v>
@@ -7890,8 +7888,8 @@
       <c r="J38" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K38" s="1" t="s">
-        <v>469</v>
+      <c r="K38" s="1">
+        <v>43</v>
       </c>
       <c r="L38" s="1">
         <v>47</v>
@@ -8012,8 +8010,8 @@
       <c r="J39" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K39" s="1" t="s">
-        <v>469</v>
+      <c r="K39" s="1">
+        <v>36</v>
       </c>
       <c r="L39" s="1">
         <v>44</v>
@@ -8134,8 +8132,8 @@
       <c r="J40" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K40" s="1" t="s">
-        <v>469</v>
+      <c r="K40" s="1">
+        <v>13</v>
       </c>
       <c r="L40" s="1">
         <v>67</v>
@@ -8256,8 +8254,8 @@
       <c r="J41" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K41" s="1" t="s">
-        <v>469</v>
+      <c r="K41" s="1">
+        <v>38</v>
       </c>
       <c r="L41" s="1">
         <v>45</v>
@@ -8378,8 +8376,8 @@
       <c r="J42" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K42" s="1" t="s">
-        <v>469</v>
+      <c r="K42" s="1">
+        <v>28</v>
       </c>
       <c r="L42" s="1">
         <v>52</v>
@@ -8500,8 +8498,8 @@
       <c r="J43" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K43" s="1" t="s">
-        <v>469</v>
+      <c r="K43" s="1">
+        <v>19</v>
       </c>
       <c r="L43" s="1">
         <v>60</v>
@@ -8622,8 +8620,8 @@
       <c r="J44" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K44" s="1" t="s">
-        <v>469</v>
+      <c r="K44" s="1">
+        <v>20</v>
       </c>
       <c r="L44" s="1">
         <v>67</v>
@@ -8744,8 +8742,8 @@
       <c r="J45" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K45" s="1" t="s">
-        <v>469</v>
+      <c r="K45" s="1">
+        <v>17</v>
       </c>
       <c r="L45" s="1">
         <v>63</v>
@@ -8866,8 +8864,8 @@
       <c r="J46" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K46" s="1" t="s">
-        <v>469</v>
+      <c r="K46" s="1">
+        <v>15</v>
       </c>
       <c r="L46" s="1">
         <v>67</v>
@@ -8988,8 +8986,8 @@
       <c r="J47" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K47" s="1" t="s">
-        <v>469</v>
+      <c r="K47" s="1">
+        <v>18</v>
       </c>
       <c r="L47" s="1">
         <v>58</v>
@@ -9110,8 +9108,8 @@
       <c r="J48" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K48" s="1" t="s">
-        <v>469</v>
+      <c r="K48" s="1">
+        <v>20</v>
       </c>
       <c r="L48" s="1">
         <v>64</v>
@@ -9232,8 +9230,8 @@
       <c r="J49" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K49" s="1" t="s">
-        <v>469</v>
+      <c r="K49" s="1">
+        <v>19</v>
       </c>
       <c r="L49" s="1">
         <v>59</v>
@@ -9354,8 +9352,8 @@
       <c r="J50" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K50" s="1" t="s">
-        <v>469</v>
+      <c r="K50" s="1">
+        <v>57</v>
       </c>
       <c r="L50" s="1">
         <v>36</v>
@@ -9479,8 +9477,8 @@
       <c r="J51" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K51" s="1" t="s">
-        <v>469</v>
+      <c r="K51" s="1">
+        <v>30</v>
       </c>
       <c r="L51" s="1">
         <v>38</v>
@@ -9601,8 +9599,8 @@
       <c r="J52" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K52" s="1" t="s">
-        <v>469</v>
+      <c r="K52" s="1">
+        <v>74</v>
       </c>
       <c r="L52" s="1">
         <v>18</v>
@@ -9723,8 +9721,8 @@
       <c r="J53" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K53" s="1" t="s">
-        <v>469</v>
+      <c r="K53" s="1">
+        <v>44</v>
       </c>
       <c r="L53" s="1">
         <v>48</v>
@@ -9845,8 +9843,8 @@
       <c r="J54" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K54" s="1" t="s">
-        <v>469</v>
+      <c r="K54" s="1">
+        <v>24</v>
       </c>
       <c r="L54" s="1">
         <v>60</v>
@@ -9967,8 +9965,8 @@
       <c r="J55" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="K55" s="1" t="s">
-        <v>469</v>
+      <c r="K55" s="1">
+        <v>64</v>
       </c>
       <c r="L55" s="1">
         <v>16</v>
@@ -10089,8 +10087,8 @@
       <c r="J56" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="K56" s="1" t="s">
-        <v>469</v>
+      <c r="K56" s="1">
+        <v>56</v>
       </c>
       <c r="L56" s="1">
         <v>24</v>
@@ -10211,8 +10209,8 @@
       <c r="J57" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K57" s="1" t="s">
-        <v>469</v>
+      <c r="K57" s="1">
+        <v>48</v>
       </c>
       <c r="L57" s="1">
         <v>40</v>
@@ -10333,8 +10331,8 @@
       <c r="J58" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K58" s="1" t="s">
-        <v>469</v>
+      <c r="K58" s="1">
+        <v>23</v>
       </c>
       <c r="L58" s="1">
         <v>53</v>
@@ -10455,8 +10453,8 @@
       <c r="J59" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K59" s="1" t="s">
-        <v>469</v>
+      <c r="K59" s="1">
+        <v>78</v>
       </c>
       <c r="L59" s="1">
         <v>16</v>
@@ -10577,8 +10575,8 @@
       <c r="J60" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K60" s="1" t="s">
-        <v>469</v>
+      <c r="K60" s="1">
+        <v>38</v>
       </c>
       <c r="L60" s="1">
         <v>34</v>
@@ -10699,8 +10697,8 @@
       <c r="J61" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K61" s="1" t="s">
-        <v>469</v>
+      <c r="K61" s="1">
+        <v>40</v>
       </c>
       <c r="L61" s="1">
         <v>50</v>
@@ -10821,8 +10819,8 @@
       <c r="J62" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K62" s="1" t="s">
-        <v>469</v>
+      <c r="K62" s="1">
+        <v>27</v>
       </c>
       <c r="L62" s="1">
         <v>62</v>
@@ -10943,8 +10941,8 @@
       <c r="J63" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K63" s="1" t="s">
-        <v>469</v>
+      <c r="K63" s="1">
+        <v>51</v>
       </c>
       <c r="L63" s="1">
         <v>44</v>
@@ -11068,8 +11066,8 @@
       <c r="J64" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K64" s="1" t="s">
-        <v>469</v>
+      <c r="K64" s="1">
+        <v>66</v>
       </c>
       <c r="L64" s="1">
         <v>18</v>
@@ -11193,8 +11191,8 @@
       <c r="J65" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K65" s="1" t="s">
-        <v>469</v>
+      <c r="K65" s="1">
+        <v>50</v>
       </c>
       <c r="L65" s="1">
         <v>42</v>
@@ -11315,8 +11313,8 @@
       <c r="J66" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K66" s="1" t="s">
-        <v>469</v>
+      <c r="K66" s="1">
+        <v>60</v>
       </c>
       <c r="L66" s="1">
         <v>30</v>
@@ -11437,8 +11435,8 @@
       <c r="J67" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K67" s="1" t="s">
-        <v>469</v>
+      <c r="K67" s="1">
+        <v>56</v>
       </c>
       <c r="L67" s="1">
         <v>39</v>
@@ -11559,8 +11557,8 @@
       <c r="J68" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K68" s="1" t="s">
-        <v>469</v>
+      <c r="K68" s="1">
+        <v>48</v>
       </c>
       <c r="L68" s="1">
         <v>40</v>
@@ -11681,8 +11679,8 @@
       <c r="J69" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K69" s="1" t="s">
-        <v>469</v>
+      <c r="K69" s="1">
+        <v>28</v>
       </c>
       <c r="L69" s="1">
         <v>58</v>
@@ -11803,8 +11801,8 @@
       <c r="J70" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K70" s="1" t="s">
-        <v>469</v>
+      <c r="K70" s="1">
+        <v>19</v>
       </c>
       <c r="L70" s="1">
         <v>68</v>
@@ -11925,8 +11923,8 @@
       <c r="J71" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K71" s="1" t="s">
-        <v>469</v>
+      <c r="K71" s="1">
+        <v>52</v>
       </c>
       <c r="L71" s="1">
         <v>43</v>
@@ -12047,8 +12045,8 @@
       <c r="J72" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K72" s="1" t="s">
-        <v>469</v>
+      <c r="K72" s="1">
+        <v>49</v>
       </c>
       <c r="L72" s="1">
         <v>47</v>
@@ -12169,8 +12167,8 @@
       <c r="J73" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K73" s="1" t="s">
-        <v>469</v>
+      <c r="K73" s="1">
+        <v>39</v>
       </c>
       <c r="L73" s="1">
         <v>53</v>
@@ -12291,8 +12289,8 @@
       <c r="J74" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K74" s="1" t="s">
-        <v>469</v>
+      <c r="K74" s="1">
+        <v>70</v>
       </c>
       <c r="L74" s="1">
         <v>24</v>
@@ -12413,8 +12411,8 @@
       <c r="J75" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K75" s="1" t="s">
-        <v>469</v>
+      <c r="K75" s="1">
+        <v>52</v>
       </c>
       <c r="L75" s="1">
         <v>39</v>
@@ -12535,8 +12533,8 @@
       <c r="J76" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K76" s="1" t="s">
-        <v>469</v>
+      <c r="K76" s="1">
+        <v>36</v>
       </c>
       <c r="L76" s="1">
         <v>48</v>
@@ -12657,8 +12655,8 @@
       <c r="J77" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K77" s="1" t="s">
-        <v>469</v>
+      <c r="K77" s="1">
+        <v>44</v>
       </c>
       <c r="L77" s="1">
         <v>44</v>
@@ -12779,8 +12777,8 @@
       <c r="J78" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K78" s="1" t="s">
-        <v>469</v>
+      <c r="K78" s="1">
+        <v>34</v>
       </c>
       <c r="L78" s="1">
         <v>54</v>
@@ -12901,8 +12899,8 @@
       <c r="J79" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K79" s="1" t="s">
-        <v>469</v>
+      <c r="K79" s="1">
+        <v>20</v>
       </c>
       <c r="L79" s="1">
         <v>58</v>
@@ -13023,8 +13021,8 @@
       <c r="J80" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K80" s="1" t="s">
-        <v>469</v>
+      <c r="K80" s="1">
+        <v>69</v>
       </c>
       <c r="L80" s="1">
         <v>27</v>
@@ -13145,8 +13143,8 @@
       <c r="J81" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K81" s="1" t="s">
-        <v>469</v>
+      <c r="K81" s="1">
+        <v>82</v>
       </c>
       <c r="L81" s="1">
         <v>14</v>
@@ -13267,8 +13265,8 @@
       <c r="J82" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K82" s="1" t="s">
-        <v>469</v>
+      <c r="K82" s="1">
+        <v>74</v>
       </c>
       <c r="L82" s="1">
         <v>18</v>
@@ -13389,8 +13387,8 @@
       <c r="J83" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K83" s="1" t="s">
-        <v>469</v>
+      <c r="K83" s="1">
+        <v>52</v>
       </c>
       <c r="L83" s="1">
         <v>32</v>
@@ -13511,8 +13509,8 @@
       <c r="J84" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K84" s="1" t="s">
-        <v>469</v>
+      <c r="K84" s="1">
+        <v>34</v>
       </c>
       <c r="L84" s="1">
         <v>50</v>
@@ -13633,8 +13631,8 @@
       <c r="J85" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K85" s="1" t="s">
-        <v>469</v>
+      <c r="K85" s="1">
+        <v>52</v>
       </c>
       <c r="L85" s="1">
         <v>40</v>
@@ -13755,8 +13753,8 @@
       <c r="J86" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K86" s="1" t="s">
-        <v>469</v>
+      <c r="K86" s="1">
+        <v>50</v>
       </c>
       <c r="L86" s="1">
         <v>39</v>
@@ -13877,8 +13875,8 @@
       <c r="J87" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K87" s="1" t="s">
-        <v>469</v>
+      <c r="K87" s="1">
+        <v>72</v>
       </c>
       <c r="L87" s="1">
         <v>24</v>
@@ -13999,8 +13997,8 @@
       <c r="J88" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K88" s="1" t="s">
-        <v>469</v>
+      <c r="K88" s="1">
+        <v>20</v>
       </c>
       <c r="L88" s="1">
         <v>64</v>
@@ -14121,8 +14119,8 @@
       <c r="J89" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K89" s="1" t="s">
-        <v>469</v>
+      <c r="K89" s="1">
+        <v>40</v>
       </c>
       <c r="L89" s="1">
         <v>52</v>
@@ -14243,8 +14241,8 @@
       <c r="J90" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K90" s="1" t="s">
-        <v>469</v>
+      <c r="K90" s="1">
+        <v>56</v>
       </c>
       <c r="L90" s="1">
         <v>36</v>
@@ -14365,8 +14363,8 @@
       <c r="J91" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K91" s="1" t="s">
-        <v>469</v>
+      <c r="K91" s="1">
+        <v>62</v>
       </c>
       <c r="L91" s="1">
         <v>28</v>
@@ -14487,8 +14485,8 @@
       <c r="J92" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="K92" s="1" t="s">
-        <v>469</v>
+      <c r="K92" s="1">
+        <v>40</v>
       </c>
       <c r="L92" s="1">
         <v>36</v>
@@ -14609,8 +14607,8 @@
       <c r="J93" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K93" s="1" t="s">
-        <v>469</v>
+      <c r="K93" s="1">
+        <v>64</v>
       </c>
       <c r="L93" s="1">
         <v>26</v>
@@ -14731,8 +14729,8 @@
       <c r="J94" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K94" s="1" t="s">
-        <v>469</v>
+      <c r="K94" s="1">
+        <v>74</v>
       </c>
       <c r="L94" s="1">
         <v>18</v>
@@ -14853,8 +14851,8 @@
       <c r="J95" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K95" s="1" t="s">
-        <v>469</v>
+      <c r="K95" s="1">
+        <v>70</v>
       </c>
       <c r="L95" s="1">
         <v>22</v>
@@ -14975,8 +14973,8 @@
       <c r="J96" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="K96" s="1" t="s">
-        <v>469</v>
+      <c r="K96" s="1">
+        <v>14</v>
       </c>
       <c r="L96" s="1">
         <v>59</v>
@@ -15097,8 +15095,8 @@
       <c r="J97" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K97" s="1" t="s">
-        <v>469</v>
+      <c r="K97" s="1">
+        <v>18</v>
       </c>
       <c r="L97" s="1">
         <v>65</v>
@@ -15219,8 +15217,8 @@
       <c r="J98" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K98" s="1" t="s">
-        <v>469</v>
+      <c r="K98" s="1">
+        <v>28</v>
       </c>
       <c r="L98" s="1">
         <v>60</v>
@@ -15341,8 +15339,8 @@
       <c r="J99" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K99" s="1" t="s">
-        <v>469</v>
+      <c r="K99" s="1">
+        <v>68</v>
       </c>
       <c r="L99" s="1">
         <v>18</v>
@@ -15463,8 +15461,8 @@
       <c r="J100" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="K100" s="1" t="s">
-        <v>469</v>
+      <c r="K100" s="1">
+        <v>5</v>
       </c>
       <c r="L100" s="1">
         <v>60</v>
@@ -15585,8 +15583,8 @@
       <c r="J101" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="K101" s="1" t="s">
-        <v>469</v>
+      <c r="K101" s="1">
+        <v>20</v>
       </c>
       <c r="L101" s="1">
         <v>62</v>
@@ -15706,222 +15704,247 @@
       <formula>COUNTIFS($D$2:$D$101,$D2,$A$2:$A$101,$A2,$E$2:$E$101,$E2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A101">
+    <cfRule type="expression" dxfId="0" priority="7">
+      <formula>AND($A2&lt;&gt;"",NOT(ISNUMBER($A2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F101">
+    <cfRule type="expression" dxfId="0" priority="8">
+      <formula>AND($F2&lt;&gt;"",ISNUMBER($F2))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G101">
+    <cfRule type="expression" dxfId="0" priority="9">
+      <formula>AND($G2&lt;&gt;"",ISNUMBER($G2))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I101">
+    <cfRule type="expression" dxfId="0" priority="10">
+      <formula>AND($I2&lt;&gt;"",NOT(ISNUMBER($I2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H101">
+    <cfRule type="expression" dxfId="0" priority="11">
+      <formula>AND($H2&lt;&gt;"",NOT(ISNUMBER($H2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K2:K101">
-    <cfRule type="expression" dxfId="1" priority="7">
+    <cfRule type="expression" dxfId="1" priority="12">
       <formula>AND(K2&lt;&gt;"",NOT(ISNUMBER(K2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L101">
-    <cfRule type="expression" dxfId="1" priority="8">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>AND(L2&lt;&gt;"",NOT(ISNUMBER(L2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M101">
-    <cfRule type="expression" dxfId="1" priority="9">
+    <cfRule type="expression" dxfId="1" priority="14">
       <formula>AND(M2&lt;&gt;"",NOT(ISNUMBER(M2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N101">
-    <cfRule type="expression" dxfId="1" priority="10">
+    <cfRule type="expression" dxfId="1" priority="15">
       <formula>AND(N2&lt;&gt;"",NOT(ISNUMBER(N2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O101">
-    <cfRule type="expression" dxfId="1" priority="11">
+    <cfRule type="expression" dxfId="1" priority="16">
       <formula>AND(O2&lt;&gt;"",NOT(ISNUMBER(O2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:P101">
-    <cfRule type="expression" dxfId="1" priority="12">
+    <cfRule type="expression" dxfId="1" priority="17">
       <formula>AND(P2&lt;&gt;"",NOT(ISNUMBER(P2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:Q101">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="1" priority="18">
       <formula>AND(Q2&lt;&gt;"",NOT(ISNUMBER(Q2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R2:R101">
-    <cfRule type="expression" dxfId="1" priority="14">
+    <cfRule type="expression" dxfId="1" priority="19">
       <formula>AND(R2&lt;&gt;"",NOT(ISNUMBER(R2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:S101">
-    <cfRule type="expression" dxfId="1" priority="15">
+    <cfRule type="expression" dxfId="1" priority="20">
       <formula>AND(S2&lt;&gt;"",NOT(ISNUMBER(S2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T2:T101">
-    <cfRule type="expression" dxfId="1" priority="16">
+    <cfRule type="expression" dxfId="1" priority="21">
       <formula>AND(T2&lt;&gt;"",NOT(ISNUMBER(T2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U2:U101">
-    <cfRule type="expression" dxfId="1" priority="17">
+    <cfRule type="expression" dxfId="1" priority="22">
       <formula>AND(U2&lt;&gt;"",NOT(ISNUMBER(U2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2:V101">
-    <cfRule type="expression" dxfId="1" priority="18">
+    <cfRule type="expression" dxfId="1" priority="23">
       <formula>AND(V2&lt;&gt;"",NOT(ISNUMBER(V2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W2:W101">
-    <cfRule type="expression" dxfId="1" priority="19">
+    <cfRule type="expression" dxfId="1" priority="24">
       <formula>AND(W2&lt;&gt;"",NOT(ISNUMBER(W2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X2:X101">
-    <cfRule type="expression" dxfId="1" priority="20">
+    <cfRule type="expression" dxfId="1" priority="25">
       <formula>AND(X2&lt;&gt;"",NOT(ISNUMBER(X2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y2:Y101">
-    <cfRule type="expression" dxfId="1" priority="21">
+    <cfRule type="expression" dxfId="1" priority="26">
       <formula>AND(Y2&lt;&gt;"",NOT(ISNUMBER(Y2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z2:Z101">
-    <cfRule type="expression" dxfId="1" priority="22">
+    <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(Z2&lt;&gt;"",NOT(ISNUMBER(Z2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA2:AA101">
-    <cfRule type="expression" dxfId="1" priority="23">
+    <cfRule type="expression" dxfId="1" priority="28">
       <formula>AND(AA2&lt;&gt;"",NOT(ISNUMBER(AA2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB2:AB101">
-    <cfRule type="expression" dxfId="1" priority="24">
+    <cfRule type="expression" dxfId="1" priority="29">
       <formula>AND(AB2&lt;&gt;"",NOT(ISNUMBER(AB2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC2:AC101">
-    <cfRule type="expression" dxfId="1" priority="25">
+    <cfRule type="expression" dxfId="1" priority="30">
       <formula>AND(AC2&lt;&gt;"",NOT(ISNUMBER(AC2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD2:AD101">
-    <cfRule type="expression" dxfId="1" priority="26">
+    <cfRule type="expression" dxfId="1" priority="31">
       <formula>AND(AD2&lt;&gt;"",NOT(ISNUMBER(AD2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE2:AE101">
-    <cfRule type="expression" dxfId="1" priority="27">
+    <cfRule type="expression" dxfId="1" priority="32">
       <formula>AND(AE2&lt;&gt;"",NOT(ISNUMBER(AE2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF2:AF101">
-    <cfRule type="expression" dxfId="1" priority="28">
+    <cfRule type="expression" dxfId="1" priority="33">
       <formula>AND(AF2&lt;&gt;"",NOT(ISNUMBER(AF2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG2:AG101">
-    <cfRule type="expression" dxfId="1" priority="29">
+    <cfRule type="expression" dxfId="1" priority="34">
       <formula>AND(AG2&lt;&gt;"",NOT(ISNUMBER(AG2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH2:AH101">
-    <cfRule type="expression" dxfId="1" priority="30">
+    <cfRule type="expression" dxfId="1" priority="35">
       <formula>AND(AH2&lt;&gt;"",NOT(ISNUMBER(AH2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI2:AI101">
-    <cfRule type="expression" dxfId="1" priority="31">
+    <cfRule type="expression" dxfId="1" priority="36">
       <formula>AND(AI2&lt;&gt;"",NOT(ISNUMBER(AI2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ2:AJ101">
-    <cfRule type="expression" dxfId="1" priority="32">
+    <cfRule type="expression" dxfId="1" priority="37">
       <formula>AND(AJ2&lt;&gt;"",NOT(ISNUMBER(AJ2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK2:AK101">
-    <cfRule type="expression" dxfId="1" priority="33">
+    <cfRule type="expression" dxfId="1" priority="38">
       <formula>AND(AK2&lt;&gt;"",NOT(ISNUMBER(AK2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL2:AL101">
-    <cfRule type="expression" dxfId="1" priority="34">
+    <cfRule type="expression" dxfId="1" priority="39">
       <formula>AND(AL2&lt;&gt;"",NOT(ISNUMBER(AL2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM2:AM101">
-    <cfRule type="expression" dxfId="1" priority="35">
+    <cfRule type="expression" dxfId="1" priority="40">
       <formula>AND(AM2&lt;&gt;"",NOT(ISNUMBER(AM2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AN2:AN101">
-    <cfRule type="expression" dxfId="1" priority="36">
+    <cfRule type="expression" dxfId="1" priority="41">
       <formula>AND(AN2&lt;&gt;"",NOT(ISNUMBER(AN2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO2:AO101">
-    <cfRule type="expression" dxfId="1" priority="37">
+    <cfRule type="expression" dxfId="1" priority="42">
       <formula>AND(AO2&lt;&gt;"",NOT(ISNUMBER(AO2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K101">
-    <cfRule type="expression" dxfId="0" priority="38">
+    <cfRule type="expression" dxfId="0" priority="43">
       <formula>K2&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K101">
-    <cfRule type="expression" dxfId="0" priority="39">
+    <cfRule type="expression" dxfId="0" priority="44">
       <formula>K2&gt;100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L101">
-    <cfRule type="expression" dxfId="0" priority="40">
+    <cfRule type="expression" dxfId="0" priority="45">
       <formula>L2&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L101">
-    <cfRule type="expression" dxfId="0" priority="41">
+    <cfRule type="expression" dxfId="0" priority="46">
       <formula>L2&gt;100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M101">
-    <cfRule type="expression" dxfId="0" priority="42">
+    <cfRule type="expression" dxfId="0" priority="47">
       <formula>M2&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M101">
-    <cfRule type="expression" dxfId="0" priority="43">
+    <cfRule type="expression" dxfId="0" priority="48">
       <formula>M2&gt;100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:M101">
-    <cfRule type="expression" dxfId="0" priority="44">
+    <cfRule type="expression" dxfId="0" priority="49">
       <formula>AND((ISNUMBER($K2)+ISNUMBER($L2)+ISNUMBER($M2))=3,OR($K2+$L2+$M2&lt;99,$K2+$L2+$M2&gt;101))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:M101">
-    <cfRule type="expression" dxfId="1" priority="45">
+    <cfRule type="expression" dxfId="1" priority="50">
       <formula>AND(ISBLANK($J2), (ISBLANK($K2)+ISBLANK($L2)+ISBLANK($M2))&gt;=2)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K101">
-    <cfRule type="expression" dxfId="1" priority="46">
+    <cfRule type="expression" dxfId="1" priority="51">
       <formula>AND(
-        ISBLANK(K2),
-        (ISBLANK(K2)+ISBLANK(L2)+ISBLANK(M2))=1
+        ISBLANK($K2),
+        (ISBLANK($K2)+ISBLANK($L2)+ISBLANK($M2))=1
       )</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L101">
-    <cfRule type="expression" dxfId="1" priority="47">
+    <cfRule type="expression" dxfId="1" priority="52">
       <formula>AND(
-        ISBLANK(L2),
-        (ISBLANK(K2)+ISBLANK(L2)+ISBLANK(M2))=1
+        ISBLANK($L2),
+        (ISBLANK($K2)+ISBLANK($L2)+ISBLANK($M2))=1
       )</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M101">
-    <cfRule type="expression" dxfId="1" priority="48">
+    <cfRule type="expression" dxfId="1" priority="53">
       <formula>AND(
-        ISBLANK(M2),
-        (ISBLANK(K2)+ISBLANK(L2)+ISBLANK(M2))=1
+        ISBLANK($M2),
+        (ISBLANK($K2)+ISBLANK($L2)+ISBLANK($M2))=1
       )</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16134,7 +16157,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>137</v>
+        <v>469</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
@@ -16218,7 +16241,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>146</v>
+        <v>470</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>172</v>
@@ -16420,6 +16443,16 @@
       <formula>COUNTIFS($D$2:$D$33,$D2,$C$2:$C$33,$C2)&gt;1</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B33">
+    <cfRule type="expression" dxfId="1" priority="5">
+      <formula>ISNA(MATCH(B2,Data!$1:$1,0))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A33">
+    <cfRule type="expression" dxfId="1" priority="6">
+      <formula>AND(A2&lt;&gt;"",ISNA(MATCH(A2,valid_groups,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -16427,7 +16460,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B100"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -16440,7 +16473,7 @@
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="20" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
@@ -16454,413 +16487,65 @@
       </c>
       <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>Non-numeric values were converted to NA (e.g., ND, &lt;1).
-Measurement columns affected:
-"sand_percent" (100 values)
-"bd_g_cm3" (3 values)
-"om_percent" (2 values)</t>
+          <t>Invalid measurement_group values: "a" and "f".
+Valid options for English:
+"Physical", "Biological", "Chemical", "Plant Essential Macro Nutrients", and "Plant Essential Micro Nutrients"</t>
         </is>
       </c>
     </row>
+  </sheetData>
+  <printOptions gridLines="1" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>Biological</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
-          <t>Texture validation skipped: "sand_percent" must be numeric.</t>
+          <t>Chemical</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="19"/>
-      <c r="B4" s="19"/>
-    </row>
     <row r="5">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Plant Essential Macro Nutrients</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="19"/>
-      <c r="B7" s="19"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="19"/>
-      <c r="B8" s="19"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19"/>
-      <c r="B9" s="19"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="19"/>
-      <c r="B10" s="19"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="19"/>
-      <c r="B13" s="19"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="19"/>
-      <c r="B14" s="19"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="19"/>
-      <c r="B16" s="19"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="19"/>
-      <c r="B17" s="19"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="19"/>
-      <c r="B18" s="19"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="19"/>
-      <c r="B19" s="19"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="19"/>
-      <c r="B21" s="19"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="19"/>
-      <c r="B22" s="19"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="19"/>
-      <c r="B24" s="19"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="19"/>
-      <c r="B25" s="19"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="19"/>
-      <c r="B34" s="19"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="19"/>
-      <c r="B35" s="19"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="19"/>
-      <c r="B36" s="19"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="19"/>
-      <c r="B39" s="19"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="19"/>
-      <c r="B40" s="19"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="19"/>
-      <c r="B41" s="19"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="19"/>
-      <c r="B42" s="19"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="19"/>
-      <c r="B43" s="19"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="19"/>
-      <c r="B44" s="19"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="19"/>
-      <c r="B45" s="19"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="19"/>
-      <c r="B46" s="19"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="19"/>
-      <c r="B47" s="19"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="19"/>
-      <c r="B48" s="19"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="19"/>
-      <c r="B49" s="19"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="19"/>
-      <c r="B50" s="19"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="19"/>
-      <c r="B51" s="19"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="19"/>
-      <c r="B52" s="19"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="19"/>
-      <c r="B53" s="19"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="19"/>
-      <c r="B54" s="19"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="19"/>
-      <c r="B55" s="19"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="19"/>
-      <c r="B56" s="19"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="19"/>
-      <c r="B57" s="19"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="19"/>
-      <c r="B58" s="19"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="19"/>
-      <c r="B59" s="19"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="19"/>
-      <c r="B60" s="19"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="19"/>
-      <c r="B61" s="19"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="19"/>
-      <c r="B62" s="19"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="19"/>
-      <c r="B63" s="19"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="19"/>
-      <c r="B64" s="19"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="19"/>
-      <c r="B65" s="19"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="19"/>
-      <c r="B66" s="19"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="19"/>
-      <c r="B67" s="19"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="19"/>
-      <c r="B68" s="19"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="19"/>
-      <c r="B69" s="19"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="19"/>
-      <c r="B70" s="19"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="19"/>
-      <c r="B71" s="19"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="19"/>
-      <c r="B72" s="19"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="19"/>
-      <c r="B73" s="19"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="19"/>
-      <c r="B74" s="19"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="19"/>
-      <c r="B75" s="19"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="19"/>
-      <c r="B76" s="19"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="19"/>
-      <c r="B77" s="19"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="19"/>
-      <c r="B78" s="19"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="19"/>
-      <c r="B79" s="19"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="19"/>
-      <c r="B80" s="19"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="19"/>
-      <c r="B81" s="19"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="19"/>
-      <c r="B82" s="19"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="19"/>
-      <c r="B83" s="19"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="19"/>
-      <c r="B84" s="19"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="19"/>
-      <c r="B85" s="19"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="19"/>
-      <c r="B86" s="19"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="19"/>
-      <c r="B87" s="19"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="19"/>
-      <c r="B88" s="19"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="19"/>
-      <c r="B89" s="19"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="19"/>
-      <c r="B90" s="19"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="19"/>
-      <c r="B91" s="19"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="19"/>
-      <c r="B92" s="19"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="19"/>
-      <c r="B93" s="19"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="19"/>
-      <c r="B94" s="19"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="19"/>
-      <c r="B95" s="19"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="19"/>
-      <c r="B96" s="19"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="19"/>
-      <c r="B97" s="19"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="19"/>
-      <c r="B98" s="19"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="19"/>
-      <c r="B99" s="19"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="19"/>
-      <c r="B100" s="19"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plant Essential Micro Nutrients</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions gridLines="1" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Add check for coordinates
</commit_message>
<xml_diff>
--- a/tests/test-files/data-issues.xlsx
+++ b/tests/test-files/data-issues.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D701B2C-02FF-4020-9E32-9243051A9ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89E2C21-3F2A-4885-83A5-3F4D552BFDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Data Dictionary" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Issues" sheetId="6" state="visible" r:id="rId4"/>
-    <sheet name="ref" sheetId="7" state="hidden" r:id="rId5"/>
+    <sheet name="Reference" sheetId="7" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="valid_groups">'ref'!$A$2:$A$5</definedName>
+    <definedName name="valid_groups">'Reference'!$A$2:$A$5</definedName>
   </definedNames>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="469">
   <si>
     <t>year</t>
   </si>
@@ -2533,18 +2533,12 @@
       <t>: Combination of abbreviation and unit be unique for each measurement.</t>
     </r>
   </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2615,6 +2609,11 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Aptos Narrow"/>
     </font>
@@ -2672,7 +2671,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2710,10 +2709,14 @@
     <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0">
@@ -3851,7 +3854,7 @@
         <v>72</v>
       </c>
       <c r="H5" s="1">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="I5" s="1">
         <v>-123</v>
@@ -4095,7 +4098,7 @@
         <v>88</v>
       </c>
       <c r="H7" s="1">
-        <v>47</v>
+        <v>-150</v>
       </c>
       <c r="I7" s="1">
         <v>-120</v>
@@ -4463,9 +4466,6 @@
       <c r="G10" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="H10" s="1">
-        <v>47</v>
-      </c>
       <c r="I10" s="1">
         <v>-119</v>
       </c>
@@ -4588,9 +4588,6 @@
       <c r="H11" s="1">
         <v>47</v>
       </c>
-      <c r="I11" s="1">
-        <v>-119</v>
-      </c>
       <c r="J11" s="1" t="s">
         <v>45</v>
       </c>
@@ -4711,7 +4708,7 @@
         <v>48</v>
       </c>
       <c r="I12" s="1">
-        <v>-123</v>
+        <v>-200</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>62</v>
@@ -5556,7 +5553,7 @@
         <v>47</v>
       </c>
       <c r="I19" s="1">
-        <v>-123</v>
+        <v>250</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>96</v>
@@ -9835,7 +9832,7 @@
         <v>55</v>
       </c>
       <c r="H54" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I54" s="1">
         <v>-117</v>
@@ -9957,7 +9954,7 @@
         <v>55</v>
       </c>
       <c r="H55" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I55" s="1">
         <v>-117</v>
@@ -10079,7 +10076,7 @@
         <v>55</v>
       </c>
       <c r="H56" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I56" s="1">
         <v>-117</v>
@@ -10201,7 +10198,7 @@
         <v>58</v>
       </c>
       <c r="H57" s="1">
-        <v>46</v>
+        <v>200</v>
       </c>
       <c r="I57" s="1">
         <v>-123</v>
@@ -10323,7 +10320,7 @@
         <v>53</v>
       </c>
       <c r="H58" s="1">
-        <v>46</v>
+        <v>200</v>
       </c>
       <c r="I58" s="1">
         <v>-123</v>
@@ -10445,7 +10442,7 @@
         <v>40</v>
       </c>
       <c r="H59" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I59" s="1">
         <v>-119</v>
@@ -10567,7 +10564,7 @@
         <v>40</v>
       </c>
       <c r="H60" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I60" s="1">
         <v>-121</v>
@@ -10689,7 +10686,7 @@
         <v>68</v>
       </c>
       <c r="H61" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I61" s="1">
         <v>-123</v>
@@ -10811,7 +10808,7 @@
         <v>55</v>
       </c>
       <c r="H62" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I62" s="1">
         <v>-118</v>
@@ -10933,7 +10930,7 @@
         <v>80</v>
       </c>
       <c r="H63" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I63" s="1">
         <v>-120</v>
@@ -11058,7 +11055,7 @@
         <v>53</v>
       </c>
       <c r="H64" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I64" s="1">
         <v>-120</v>
@@ -11183,7 +11180,7 @@
         <v>53</v>
       </c>
       <c r="H65" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I65" s="1">
         <v>-117</v>
@@ -11305,7 +11302,7 @@
         <v>53</v>
       </c>
       <c r="H66" s="1">
-        <v>48</v>
+        <v>200</v>
       </c>
       <c r="I66" s="1">
         <v>-117</v>
@@ -11427,7 +11424,7 @@
         <v>47</v>
       </c>
       <c r="H67" s="1">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="I67" s="1">
         <v>-122</v>
@@ -11549,7 +11546,7 @@
         <v>47</v>
       </c>
       <c r="H68" s="1">
-        <v>49</v>
+        <v>200</v>
       </c>
       <c r="I68" s="1">
         <v>-123</v>
@@ -11671,7 +11668,7 @@
         <v>78</v>
       </c>
       <c r="H69" s="1">
-        <v>49</v>
+        <v>200</v>
       </c>
       <c r="I69" s="1">
         <v>-123</v>
@@ -11793,7 +11790,7 @@
         <v>80</v>
       </c>
       <c r="H70" s="1">
-        <v>46</v>
+        <v>200</v>
       </c>
       <c r="I70" s="1">
         <v>-118</v>
@@ -11915,7 +11912,7 @@
         <v>72</v>
       </c>
       <c r="H71" s="1">
-        <v>49</v>
+        <v>200</v>
       </c>
       <c r="I71" s="1">
         <v>-122</v>
@@ -15948,6 +15945,21 @@
       )</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H101">
+    <cfRule type="expression" dxfId="0" priority="54">
+      <formula>AND(H2&lt;&gt;"",OR(H2&lt;-90,H2&gt;90))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I101">
+    <cfRule type="expression" dxfId="0" priority="55">
+      <formula>AND(I2&lt;&gt;"",OR(I2&lt;-180,I2&gt;180))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:I101">
+    <cfRule type="expression" dxfId="0" priority="56">
+      <formula>AND(OR(H2="",I2=""),NOT(AND(H2="",I2="")))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -16157,7 +16169,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>469</v>
+        <v>137</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
@@ -16241,7 +16253,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>470</v>
+        <v>146</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>172</v>
@@ -16460,7 +16472,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -16468,28 +16480,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="19" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>latitude has values outside valid range (-90 to 90) for: "22-TNV09-02", "22-IIJ07-02", "23-FLS08-04", …, "23-VRD07-01", and "23-XJO04-02".</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="B3" s="19" t="inlineStr">
+        <is>
+          <t>longitude has values outside valid range (-180 to 180) for: "22-FKH06-08" and "22-OWZ06-02".</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>Invalid measurement_group values: "a" and "f".
-Valid options for English:
-"Physical", "Biological", "Chemical", "Plant Essential Macro Nutrients", and "Plant Essential Micro Nutrients"</t>
+          <t>Incomplete coordinate pairs: one of latitude or longitude is missing for: "22-YYF05-02" and "22-OIO04-05".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Condense subissues into one group
</commit_message>
<xml_diff>
--- a/tests/test-files/data-issues.xlsx
+++ b/tests/test-files/data-issues.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89E2C21-3F2A-4885-83A5-3F4D552BFDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E561B97-AC71-4066-9E52-D81EC835D019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" state="visible" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="448">
   <si>
     <t>year</t>
   </si>
@@ -410,9 +410,6 @@
     <t>Farm 123</t>
   </si>
   <si>
-    <t>Farm 035</t>
-  </si>
-  <si>
     <t>column_name</t>
   </si>
   <si>
@@ -437,9 +434,6 @@
     <t>mg/kg/day</t>
   </si>
   <si>
-    <t>POXC</t>
-  </si>
-  <si>
     <t>ppm</t>
   </si>
   <si>
@@ -587,18 +581,12 @@
     <t>22-AZJ01-02</t>
   </si>
   <si>
-    <t>22-CHP09-01</t>
-  </si>
-  <si>
     <t>Farm 021</t>
   </si>
   <si>
     <t>CHP09</t>
   </si>
   <si>
-    <t>22-CHP09-03</t>
-  </si>
-  <si>
     <t>22-CNA08-01</t>
   </si>
   <si>
@@ -632,9 +620,6 @@
     <t>DJA05</t>
   </si>
   <si>
-    <t>22-DME06-01</t>
-  </si>
-  <si>
     <t>DME06</t>
   </si>
   <si>
@@ -656,9 +641,6 @@
     <t>EYT03</t>
   </si>
   <si>
-    <t>22-FKH06-08</t>
-  </si>
-  <si>
     <t>Farm 015</t>
   </si>
   <si>
@@ -674,15 +656,6 @@
     <t>FSD09</t>
   </si>
   <si>
-    <t>22-GBP03-04</t>
-  </si>
-  <si>
-    <t>GBP03</t>
-  </si>
-  <si>
-    <t>22-GBP03-07</t>
-  </si>
-  <si>
     <t>Field 07</t>
   </si>
   <si>
@@ -701,9 +674,6 @@
     <t>IIJ07</t>
   </si>
   <si>
-    <t>22-JLB06-01</t>
-  </si>
-  <si>
     <t>JLB06</t>
   </si>
   <si>
@@ -731,15 +701,9 @@
     <t>LUB02</t>
   </si>
   <si>
-    <t>22-MNU07-02</t>
-  </si>
-  <si>
     <t>MNU07</t>
   </si>
   <si>
-    <t>22-NGJ05-03</t>
-  </si>
-  <si>
     <t>NGJ05</t>
   </si>
   <si>
@@ -752,15 +716,9 @@
     <t>NHF04</t>
   </si>
   <si>
-    <t>22-NSO08-01</t>
-  </si>
-  <si>
     <t>NSO08</t>
   </si>
   <si>
-    <t>22-OIO04-05</t>
-  </si>
-  <si>
     <t>OIO04</t>
   </si>
   <si>
@@ -770,9 +728,6 @@
     <t>OSN03</t>
   </si>
   <si>
-    <t>22-OWZ06-02</t>
-  </si>
-  <si>
     <t>OWZ06</t>
   </si>
   <si>
@@ -785,9 +740,6 @@
     <t>PBO07</t>
   </si>
   <si>
-    <t>22-QWK07-01</t>
-  </si>
-  <si>
     <t>Farm 029</t>
   </si>
   <si>
@@ -812,9 +764,6 @@
     <t>UGU06</t>
   </si>
   <si>
-    <t>22-UGU06-02</t>
-  </si>
-  <si>
     <t>22-UYH07-04</t>
   </si>
   <si>
@@ -839,24 +788,15 @@
     <t>WDX03</t>
   </si>
   <si>
-    <t>22-WNN06-03</t>
-  </si>
-  <si>
     <t>Farm 055</t>
   </si>
   <si>
     <t>WNN06</t>
   </si>
   <si>
-    <t>22-XTO07-03</t>
-  </si>
-  <si>
     <t>XTO07</t>
   </si>
   <si>
-    <t>22-YGV09-02</t>
-  </si>
-  <si>
     <t>Farm 034</t>
   </si>
   <si>
@@ -888,9 +828,6 @@
   </si>
   <si>
     <t>22-YUM02-05</t>
-  </si>
-  <si>
-    <t>22-YYF05-02</t>
   </si>
   <si>
     <t>YYF05</t>
@@ -2538,7 +2475,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2612,11 +2549,6 @@
       <color rgb="FF9C0006"/>
       <name val="Aptos Narrow"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2671,7 +2603,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2709,14 +2641,10 @@
     <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0">
@@ -3049,12 +2977,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>422</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>426</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
@@ -3062,227 +2990,227 @@
     </row>
     <row r="4" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>425</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>427</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>428</v>
+        <v>407</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>429</v>
+        <v>408</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>430</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>461</v>
+        <v>440</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>431</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>432</v>
+        <v>411</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>433</v>
+        <v>412</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>434</v>
+        <v>413</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>435</v>
+        <v>414</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>423</v>
+        <v>402</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>436</v>
+        <v>415</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
-        <v>463</v>
+        <v>442</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>437</v>
+        <v>416</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>438</v>
+        <v>417</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>439</v>
+        <v>418</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
-        <v>440</v>
+        <v>419</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
-        <v>441</v>
+        <v>420</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>442</v>
+        <v>421</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>443</v>
+        <v>422</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
-        <v>444</v>
+        <v>423</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
-        <v>445</v>
+        <v>424</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
-        <v>446</v>
+        <v>425</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
-        <v>447</v>
+        <v>426</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
-        <v>464</v>
+        <v>443</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>467</v>
+        <v>446</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
-        <v>448</v>
+        <v>427</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
-        <v>449</v>
+        <v>428</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
-        <v>450</v>
+        <v>429</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
-        <v>451</v>
+        <v>430</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
-        <v>452</v>
+        <v>431</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
-        <v>453</v>
+        <v>432</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
-        <v>454</v>
+        <v>433</v>
       </c>
     </row>
     <row r="42" spans="1:1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9" t="s">
-        <v>462</v>
+        <v>441</v>
       </c>
     </row>
     <row r="44" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>424</v>
+        <v>403</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>455</v>
+        <v>434</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>465</v>
+        <v>444</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="10" t="s">
-        <v>456</v>
+        <v>435</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
-        <v>457</v>
+        <v>436</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
-        <v>458</v>
+        <v>437</v>
       </c>
     </row>
     <row r="50" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>466</v>
+        <v>445</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
-        <v>459</v>
+        <v>438</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
-        <v>460</v>
+        <v>439</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>468</v>
+        <v>447</v>
       </c>
     </row>
   </sheetData>
@@ -3399,7 +3327,7 @@
         <v>11</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>27</v>
@@ -3426,10 +3354,10 @@
         <v>26</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="AE1" s="1" t="s">
         <v>32</v>
@@ -3470,13 +3398,13 @@
         <v>2022</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>117</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>242</v>
+        <v>228</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>38</v>
@@ -3592,13 +3520,13 @@
         <v>2022</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>42</v>
@@ -3714,13 +3642,10 @@
         <v>2022</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>109</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>252</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>38</v>
@@ -3836,13 +3761,13 @@
         <v>2022</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>109</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>42</v>
@@ -3854,7 +3779,7 @@
         <v>72</v>
       </c>
       <c r="H5" s="1">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="I5" s="1">
         <v>-123</v>
@@ -3958,13 +3883,13 @@
         <v>2022</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>103</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>38</v>
@@ -4080,13 +4005,13 @@
         <v>2022</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>42</v>
@@ -4098,7 +4023,7 @@
         <v>88</v>
       </c>
       <c r="H7" s="1">
-        <v>-150</v>
+        <v>47</v>
       </c>
       <c r="I7" s="1">
         <v>-120</v>
@@ -4202,13 +4127,13 @@
         <v>2022</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>38</v>
@@ -4323,14 +4248,11 @@
       <c r="A9" s="1">
         <v>2022</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>257</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>42</v>
@@ -4448,14 +4370,11 @@
       <c r="A10" s="1">
         <v>2022</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>283</v>
-      </c>
       <c r="C10" s="1" t="s">
         <v>119</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>284</v>
+        <v>263</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>42</v>
@@ -4465,6 +4384,9 @@
       </c>
       <c r="G10" s="1" t="s">
         <v>80</v>
+      </c>
+      <c r="H10" s="1">
+        <v>47</v>
       </c>
       <c r="I10" s="1">
         <v>-119</v>
@@ -4567,14 +4489,11 @@
       <c r="A11" s="1">
         <v>2022</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>239</v>
-      </c>
       <c r="C11" s="1" t="s">
         <v>111</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>89</v>
@@ -4587,6 +4506,9 @@
       </c>
       <c r="H11" s="1">
         <v>47</v>
+      </c>
+      <c r="I11" s="1">
+        <v>-119</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>45</v>
@@ -4686,14 +4608,11 @@
       <c r="A12" s="1">
         <v>2022</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>71</v>
@@ -4708,7 +4627,7 @@
         <v>48</v>
       </c>
       <c r="I12" s="1">
-        <v>-200</v>
+        <v>-123</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>62</v>
@@ -4808,14 +4727,11 @@
       <c r="A13" s="1">
         <v>2022</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>197</v>
-      </c>
       <c r="C13" s="1" t="s">
         <v>81</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>38</v>
@@ -4930,14 +4846,11 @@
       <c r="A14" s="1">
         <v>2022</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>38</v>
@@ -5049,14 +4962,11 @@
       <c r="A15" s="1">
         <v>2022</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="C15" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>50</v>
@@ -5171,14 +5081,11 @@
       <c r="A16" s="1">
         <v>2022</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>220</v>
-      </c>
       <c r="C16" s="1" t="s">
         <v>116</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>38</v>
@@ -5293,14 +5200,11 @@
       <c r="A17" s="1">
         <v>2022</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>237</v>
-      </c>
       <c r="C17" s="1" t="s">
         <v>92</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>238</v>
+        <v>225</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>38</v>
@@ -5412,14 +5316,11 @@
       <c r="A18" s="1">
         <v>2022</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>248</v>
-      </c>
       <c r="C18" s="1" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>38</v>
@@ -5531,14 +5432,11 @@
       <c r="A19" s="1">
         <v>2022</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>243</v>
-      </c>
       <c r="C19" s="1" t="s">
         <v>94</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>42</v>
@@ -5553,7 +5451,7 @@
         <v>47</v>
       </c>
       <c r="I19" s="1">
-        <v>250</v>
+        <v>-123</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>96</v>
@@ -5653,14 +5551,11 @@
       <c r="A20" s="1">
         <v>2022</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>232</v>
-      </c>
       <c r="C20" s="1" t="s">
         <v>114</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>50</v>
@@ -5775,14 +5670,11 @@
       <c r="A21" s="1">
         <v>2022</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>271</v>
-      </c>
       <c r="C21" s="1" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>42</v>
@@ -5897,15 +5789,6 @@
       <c r="A22" s="1">
         <v>2022</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>212</v>
-      </c>
       <c r="E22" s="1" t="s">
         <v>75</v>
       </c>
@@ -6019,17 +5902,8 @@
       <c r="A23" s="1">
         <v>2022</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>212</v>
-      </c>
       <c r="E23" s="1" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>39</v>
@@ -6141,14 +6015,11 @@
       <c r="A24" s="1">
         <v>2022</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>269</v>
-      </c>
       <c r="C24" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>50</v>
@@ -6263,14 +6134,11 @@
       <c r="A25" s="1">
         <v>2022</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>230</v>
-      </c>
       <c r="C25" s="1" t="s">
         <v>121</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>42</v>
@@ -6388,14 +6256,11 @@
       <c r="A26" s="1">
         <v>2022</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>266</v>
-      </c>
       <c r="C26" s="1" t="s">
-        <v>267</v>
+        <v>249</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>50</v>
@@ -6511,13 +6376,13 @@
         <v>2022</v>
       </c>
       <c r="B27" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>38</v>
@@ -6633,13 +6498,13 @@
         <v>2022</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>42</v>
@@ -6755,13 +6620,13 @@
         <v>2022</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>70</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>42</v>
@@ -6877,13 +6742,13 @@
         <v>2022</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>107</v>
@@ -7002,13 +6867,13 @@
         <v>2022</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>113</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>75</v>
@@ -7124,13 +6989,13 @@
         <v>2022</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>74</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>75</v>
@@ -7249,16 +7114,13 @@
         <v>2022</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>108</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>75</v>
+        <v>261</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>79</v>
@@ -7371,13 +7233,13 @@
         <v>2022</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>108</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>89</v>
@@ -7493,13 +7355,13 @@
         <v>2022</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>38</v>
@@ -7615,13 +7477,13 @@
         <v>2022</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>42</v>
@@ -7737,13 +7599,13 @@
         <v>2022</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>38</v>
@@ -7859,13 +7721,13 @@
         <v>2022</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>38</v>
@@ -7981,13 +7843,13 @@
         <v>2022</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>83</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>38</v>
@@ -8103,13 +7965,13 @@
         <v>2022</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>38</v>
@@ -8225,13 +8087,13 @@
         <v>2022</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>99</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>38</v>
@@ -8347,13 +8209,13 @@
         <v>2022</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>42</v>
@@ -8469,13 +8331,13 @@
         <v>2022</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>38</v>
@@ -8591,13 +8453,13 @@
         <v>2022</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>42</v>
@@ -8713,13 +8575,13 @@
         <v>2022</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>42</v>
@@ -8835,13 +8697,13 @@
         <v>2022</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>50</v>
@@ -8957,13 +8819,13 @@
         <v>2022</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>42</v>
@@ -9079,13 +8941,13 @@
         <v>2022</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>38</v>
@@ -9201,13 +9063,13 @@
         <v>2022</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>118</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>38</v>
@@ -9323,13 +9185,13 @@
         <v>2023</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>343</v>
+        <v>322</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>344</v>
+        <v>323</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>345</v>
+        <v>324</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>75</v>
@@ -9448,13 +9310,13 @@
         <v>2023</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>290</v>
+        <v>269</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>84</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>291</v>
+        <v>270</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>50</v>
@@ -9570,13 +9432,13 @@
         <v>2023</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>331</v>
+        <v>310</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>332</v>
+        <v>311</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>333</v>
+        <v>312</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>107</v>
@@ -9692,13 +9554,13 @@
         <v>2023</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>308</v>
+        <v>287</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>105</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>309</v>
+        <v>288</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>42</v>
@@ -9814,13 +9676,13 @@
         <v>2023</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>304</v>
+        <v>283</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>305</v>
+        <v>284</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>306</v>
+        <v>285</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>75</v>
@@ -9832,7 +9694,7 @@
         <v>55</v>
       </c>
       <c r="H54" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I54" s="1">
         <v>-117</v>
@@ -9936,13 +9798,13 @@
         <v>2023</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>307</v>
+        <v>286</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>75</v>
@@ -9954,7 +9816,7 @@
         <v>55</v>
       </c>
       <c r="H55" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I55" s="1">
         <v>-117</v>
@@ -10058,13 +9920,13 @@
         <v>2023</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>318</v>
+        <v>297</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>319</v>
+        <v>298</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>320</v>
+        <v>299</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>50</v>
@@ -10076,7 +9938,7 @@
         <v>55</v>
       </c>
       <c r="H56" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I56" s="1">
         <v>-117</v>
@@ -10180,13 +10042,13 @@
         <v>2023</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>292</v>
+        <v>271</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>63</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>293</v>
+        <v>272</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>38</v>
@@ -10198,7 +10060,7 @@
         <v>58</v>
       </c>
       <c r="H57" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I57" s="1">
         <v>-123</v>
@@ -10302,13 +10164,13 @@
         <v>2023</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>338</v>
+        <v>317</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>86</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>339</v>
+        <v>318</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>38</v>
@@ -10320,7 +10182,7 @@
         <v>53</v>
       </c>
       <c r="H58" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I58" s="1">
         <v>-123</v>
@@ -10424,13 +10286,13 @@
         <v>2023</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>324</v>
+        <v>303</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>122</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>325</v>
+        <v>304</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>42</v>
@@ -10442,7 +10304,7 @@
         <v>40</v>
       </c>
       <c r="H59" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I59" s="1">
         <v>-119</v>
@@ -10546,13 +10408,13 @@
         <v>2023</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>346</v>
+        <v>325</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>347</v>
+        <v>326</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>348</v>
+        <v>327</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>38</v>
@@ -10564,7 +10426,7 @@
         <v>40</v>
       </c>
       <c r="H60" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I60" s="1">
         <v>-121</v>
@@ -10668,13 +10530,13 @@
         <v>2023</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>312</v>
+        <v>291</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>313</v>
+        <v>292</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>314</v>
+        <v>293</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>42</v>
@@ -10686,7 +10548,7 @@
         <v>68</v>
       </c>
       <c r="H61" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I61" s="1">
         <v>-123</v>
@@ -10790,13 +10652,13 @@
         <v>2023</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>298</v>
+        <v>277</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>299</v>
+        <v>278</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>300</v>
+        <v>279</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>42</v>
@@ -10808,7 +10670,7 @@
         <v>55</v>
       </c>
       <c r="H62" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I62" s="1">
         <v>-118</v>
@@ -10912,13 +10774,13 @@
         <v>2023</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>301</v>
+        <v>280</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>98</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>302</v>
+        <v>281</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>38</v>
@@ -10930,7 +10792,7 @@
         <v>80</v>
       </c>
       <c r="H63" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I63" s="1">
         <v>-120</v>
@@ -11037,13 +10899,13 @@
         <v>2023</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>303</v>
+        <v>282</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>98</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>302</v>
+        <v>281</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>50</v>
@@ -11055,7 +10917,7 @@
         <v>53</v>
       </c>
       <c r="H64" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I64" s="1">
         <v>-120</v>
@@ -11162,13 +11024,13 @@
         <v>2023</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>321</v>
+        <v>300</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>322</v>
+        <v>301</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>38</v>
@@ -11180,7 +11042,7 @@
         <v>53</v>
       </c>
       <c r="H65" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I65" s="1">
         <v>-117</v>
@@ -11284,13 +11146,13 @@
         <v>2023</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>323</v>
+        <v>302</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>322</v>
+        <v>301</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>50</v>
@@ -11302,7 +11164,7 @@
         <v>53</v>
       </c>
       <c r="H66" s="1">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="I66" s="1">
         <v>-117</v>
@@ -11406,13 +11268,13 @@
         <v>2023</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>315</v>
+        <v>294</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>316</v>
+        <v>295</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>317</v>
+        <v>296</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>42</v>
@@ -11424,7 +11286,7 @@
         <v>47</v>
       </c>
       <c r="H67" s="1">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="I67" s="1">
         <v>-122</v>
@@ -11528,13 +11390,13 @@
         <v>2023</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>328</v>
+        <v>307</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>329</v>
+        <v>308</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>330</v>
+        <v>309</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>38</v>
@@ -11546,7 +11408,7 @@
         <v>47</v>
       </c>
       <c r="H68" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I68" s="1">
         <v>-123</v>
@@ -11650,13 +11512,13 @@
         <v>2023</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>288</v>
+        <v>267</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>289</v>
+        <v>268</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>38</v>
@@ -11668,7 +11530,7 @@
         <v>78</v>
       </c>
       <c r="H69" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I69" s="1">
         <v>-123</v>
@@ -11772,25 +11634,25 @@
         <v>2023</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>334</v>
+        <v>313</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>335</v>
+        <v>314</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>337</v>
+        <v>316</v>
       </c>
       <c r="G70" s="1" t="s">
         <v>80</v>
       </c>
       <c r="H70" s="1">
-        <v>200</v>
+        <v>46</v>
       </c>
       <c r="I70" s="1">
         <v>-118</v>
@@ -11894,13 +11756,13 @@
         <v>2023</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>112</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>341</v>
+        <v>320</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>42</v>
@@ -11912,7 +11774,7 @@
         <v>72</v>
       </c>
       <c r="H71" s="1">
-        <v>200</v>
+        <v>49</v>
       </c>
       <c r="I71" s="1">
         <v>-122</v>
@@ -12016,13 +11878,13 @@
         <v>2023</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>342</v>
+        <v>321</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>112</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>341</v>
+        <v>320</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>50</v>
@@ -12138,13 +12000,13 @@
         <v>2023</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>310</v>
+        <v>289</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>76</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>311</v>
+        <v>290</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>42</v>
@@ -12260,13 +12122,13 @@
         <v>2023</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>294</v>
+        <v>273</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>295</v>
+        <v>274</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>296</v>
+        <v>275</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>42</v>
@@ -12382,13 +12244,13 @@
         <v>2023</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>297</v>
+        <v>276</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>295</v>
+        <v>274</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>296</v>
+        <v>275</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>75</v>
@@ -12504,13 +12366,13 @@
         <v>2023</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>326</v>
+        <v>305</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>87</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>327</v>
+        <v>306</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>42</v>
@@ -12626,13 +12488,13 @@
         <v>2023</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>285</v>
+        <v>264</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>286</v>
+        <v>265</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>287</v>
+        <v>266</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>38</v>
@@ -12748,13 +12610,13 @@
         <v>2024</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>375</v>
+        <v>354</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>105</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>309</v>
+        <v>288</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>89</v>
@@ -12870,13 +12732,13 @@
         <v>2024</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>367</v>
+        <v>346</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>107</v>
@@ -12992,22 +12854,22 @@
         <v>2024</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>376</v>
+        <v>355</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>377</v>
+        <v>356</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>378</v>
+        <v>357</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>379</v>
+        <v>358</v>
       </c>
       <c r="H80" s="1">
         <v>48</v>
@@ -13114,19 +12976,19 @@
         <v>2024</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>356</v>
+        <v>335</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>357</v>
+        <v>336</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>358</v>
+        <v>337</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="G81" s="1" t="s">
         <v>80</v>
@@ -13236,19 +13098,19 @@
         <v>2024</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>410</v>
+        <v>389</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>411</v>
+        <v>390</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>412</v>
+        <v>391</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>42</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>359</v>
+        <v>338</v>
       </c>
       <c r="G82" s="1" t="s">
         <v>65</v>
@@ -13358,19 +13220,19 @@
         <v>2024</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>393</v>
+        <v>372</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>394</v>
+        <v>373</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>395</v>
+        <v>374</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>352</v>
+        <v>331</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>80</v>
@@ -13480,19 +13342,19 @@
         <v>2024</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>349</v>
+        <v>328</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>350</v>
+        <v>329</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>351</v>
+        <v>330</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>42</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>352</v>
+        <v>331</v>
       </c>
       <c r="G84" s="1" t="s">
         <v>80</v>
@@ -13602,13 +13464,13 @@
         <v>2024</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>372</v>
+        <v>351</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>373</v>
+        <v>352</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>374</v>
+        <v>353</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>89</v>
@@ -13724,13 +13586,13 @@
         <v>2024</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>380</v>
+        <v>359</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>381</v>
+        <v>360</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>382</v>
+        <v>361</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>38</v>
@@ -13846,13 +13708,13 @@
         <v>2024</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>390</v>
+        <v>369</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>391</v>
+        <v>370</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>392</v>
+        <v>371</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>50</v>
@@ -13968,19 +13830,19 @@
         <v>2024</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>406</v>
+        <v>385</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>407</v>
+        <v>386</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>408</v>
+        <v>387</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>409</v>
+        <v>388</v>
       </c>
       <c r="G88" s="1" t="s">
         <v>55</v>
@@ -14090,13 +13952,13 @@
         <v>2024</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>413</v>
+        <v>392</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>414</v>
+        <v>393</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>415</v>
+        <v>394</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>38</v>
@@ -14212,19 +14074,19 @@
         <v>2024</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>416</v>
+        <v>395</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>417</v>
+        <v>396</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>418</v>
+        <v>397</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>386</v>
+        <v>365</v>
       </c>
       <c r="G90" s="1" t="s">
         <v>53</v>
@@ -14334,22 +14196,22 @@
         <v>2024</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>383</v>
+        <v>362</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>384</v>
+        <v>363</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>385</v>
+        <v>364</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>42</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>386</v>
+        <v>365</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>379</v>
+        <v>358</v>
       </c>
       <c r="H91" s="1">
         <v>48</v>
@@ -14456,13 +14318,13 @@
         <v>2024</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>396</v>
+        <v>375</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>397</v>
+        <v>376</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>398</v>
+        <v>377</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>38</v>
@@ -14578,13 +14440,13 @@
         <v>2024</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>365</v>
+        <v>344</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>366</v>
+        <v>345</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>38</v>
@@ -14700,13 +14562,13 @@
         <v>2024</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>387</v>
+        <v>366</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>388</v>
+        <v>367</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>389</v>
+        <v>368</v>
       </c>
       <c r="E94" s="1" t="s">
         <v>38</v>
@@ -14822,13 +14684,13 @@
         <v>2024</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>353</v>
+        <v>332</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>354</v>
+        <v>333</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>355</v>
+        <v>334</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>38</v>
@@ -14944,19 +14806,19 @@
         <v>2024</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>360</v>
+        <v>339</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>361</v>
+        <v>340</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>362</v>
+        <v>341</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>363</v>
+        <v>342</v>
       </c>
       <c r="G96" s="1" t="s">
         <v>53</v>
@@ -15066,19 +14928,19 @@
         <v>2024</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>399</v>
+        <v>378</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>400</v>
+        <v>379</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>401</v>
+        <v>380</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>38</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>402</v>
+        <v>381</v>
       </c>
       <c r="G97" s="1" t="s">
         <v>40</v>
@@ -15188,13 +15050,13 @@
         <v>2024</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>419</v>
+        <v>398</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>420</v>
+        <v>399</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>421</v>
+        <v>400</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>42</v>
@@ -15310,13 +15172,13 @@
         <v>2024</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>368</v>
+        <v>347</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>369</v>
+        <v>348</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>370</v>
+        <v>349</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>38</v>
@@ -15432,13 +15294,13 @@
         <v>2024</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>371</v>
+        <v>350</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>369</v>
+        <v>348</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>370</v>
+        <v>349</v>
       </c>
       <c r="E100" s="1" t="s">
         <v>75</v>
@@ -15554,13 +15416,13 @@
         <v>2024</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>403</v>
+        <v>382</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>404</v>
+        <v>383</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>405</v>
+        <v>384</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>38</v>
@@ -15979,60 +15841,60 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" t="s">
         <v>125</v>
-      </c>
-      <c r="D1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>30</v>
@@ -16041,396 +15903,390 @@
         <v>85</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>132</v>
-      </c>
       <c r="D11" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>137</v>
-      </c>
       <c r="B14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>148</v>
-      </c>
       <c r="D21" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -16480,50 +16336,56 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="19" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="B2" s="19" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
-          <t>latitude has values outside valid range (-90 to 90) for: "22-TNV09-02", "22-IIJ07-02", "23-FLS08-04", …, "23-VRD07-01", and "23-XJO04-02".</t>
+          <t>Data has missing values in required columns:
+sample_id: 18 missing values
+producer_id: 3 missing values
+field_id: 1 missing value</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
-          <t>longitude has values outside valid range (-180 to 180) for: "22-FKH06-08" and "22-OWZ06-02".</t>
+          <t>Data Dictionary has missing values in required columns:
+measurement_group: 1 missing value
+abbr: 1 missing value</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>warning</t>
+          <t>error</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Incomplete coordinate pairs: one of latitude or longitude is missing for: "22-YYF05-02" and "22-OIO04-05".</t>
+          <t>Data has duplicate values:
+sample_id: NA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add guidance as to what errors/warnings mean to issues.xlsx
</commit_message>
<xml_diff>
--- a/tests/test-files/data-issues.xlsx
+++ b/tests/test-files/data-issues.xlsx
@@ -2544,7 +2544,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2608,6 +2608,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <i val="1"/>
+      <sz val="11"/>
+      <color rgb="FF595959"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2656,7 +2662,7 @@
       </bottom>
     </border>
     <border>
-      <right style="thin">
+      <right style="none">
         <color rgb="FF000000"/>
       </right>
       <top style="thin">
@@ -2672,7 +2678,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2707,16 +2713,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf applyFont="1" borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
-    <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
-    <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0"/>
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
-    <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="9" numFmtId="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0">
+    <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
+    <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -16480,32 +16481,48 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="8.711"/>
-    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="184.711"/>
+    <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" hidden="false" width="120.711"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Errors must be corrected before proceeding.</t>
+        </is>
+      </c>
+      <c r="B1" s="13"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Warnings indicate potential issues. Processing can continue, but review is recommended.</t>
+        </is>
+      </c>
+      <c r="B2" s="13"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B1" s="19" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Message</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Invalid measurement_group values: "a" and "f".
 Valid options for English:

</xml_diff>

<commit_message>
Use same style as CF for issue rows
</commit_message>
<xml_diff>
--- a/tests/test-files/data-issues.xlsx
+++ b/tests/test-files/data-issues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jryan\Documents\R\projects\soils\tests\test-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D701B2C-02FF-4020-9E32-9243051A9ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AFB1B0D-AF4A-4670-8696-BD164EA67AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="5" state="visible" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="469">
   <si>
     <t>year</t>
   </si>
@@ -2533,18 +2533,12 @@
       <t>: Combination of abbreviation and unit be unique for each measurement.</t>
     </r>
   </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2621,19 +2615,38 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -2672,13 +2685,51 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <top style="thin"/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="none">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin"/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf applyAlignment="0" applyBorder="0" applyFill="1" applyFont="1" applyNumberFormat="0" applyProtection="0" fillId="2" fontId="11"/>
+    <xf applyAlignment="0" applyBorder="0" applyFill="1" applyFont="1" applyNumberFormat="0" applyProtection="0" fillId="3" fontId="12"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -2716,15 +2767,47 @@
     <xf applyFont="1" borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="2" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
     <xf applyBorder="1" applyFont="1" borderId="3" fillId="0" fontId="10" numFmtId="0" xfId="0"/>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0"/>
-    <xf applyFont="1" borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0">
+    <xf borderId="0" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf applyBorder="1" borderId="4" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf applyBorder="1" borderId="5" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf applyBorder="1" borderId="6" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf applyBorder="1" borderId="7" fillId="2" fontId="11" numFmtId="0" xfId="3"/>
+    <xf borderId="0" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="5" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="6" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="7" fillId="3" fontId="12" numFmtId="0" xfId="4"/>
+    <xf applyBorder="1" borderId="4" fillId="2" fontId="11" numFmtId="0" xfId="3">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="6" fillId="2" fontId="11" numFmtId="0" xfId="3">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="4" fillId="3" fontId="12" numFmtId="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="6" fillId="3" fontId="12" numFmtId="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="5" fillId="2" fontId="11" numFmtId="0" xfId="3">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="7" fillId="2" fontId="11" numFmtId="0" xfId="3">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="5" fillId="3" fontId="12" numFmtId="0" xfId="4">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" borderId="7" fillId="3" fontId="12" numFmtId="0" xfId="4">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{CDD386B2-9C7B-4451-A208-3982823DA7A1}"/>
     <cellStyle name="Normal 2 2" xfId="2" xr:uid="{CF77DDE4-DEBD-467F-927F-6AADE9C385D4}"/>
+    <cellStyle name="Bad" xfId="3" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="4" builtinId="28"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -3495,7 +3578,7 @@
         <v>41</v>
       </c>
       <c r="K2" s="1">
-        <v>29</v>
+        <v>101</v>
       </c>
       <c r="L2" s="1">
         <v>36</v>
@@ -3985,9 +4068,6 @@
       <c r="K6" s="1">
         <v>28</v>
       </c>
-      <c r="L6" s="1">
-        <v>43</v>
-      </c>
       <c r="M6" s="1">
         <v>29</v>
       </c>
@@ -4352,7 +4432,7 @@
         <v>71</v>
       </c>
       <c r="L9" s="1">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="M9" s="1">
         <v>2</v>
@@ -4595,12 +4675,6 @@
       <c r="J11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K11" s="1">
-        <v>53</v>
-      </c>
-      <c r="L11" s="1">
-        <v>41</v>
-      </c>
       <c r="M11" s="1">
         <v>6</v>
       </c>
@@ -5080,15 +5154,6 @@
       <c r="J15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="K15" s="1">
-        <v>61</v>
-      </c>
-      <c r="L15" s="1">
-        <v>33</v>
-      </c>
-      <c r="M15" s="1">
-        <v>6</v>
-      </c>
       <c r="N15" s="1">
         <v>0.55000000000000004</v>
       </c>
@@ -5559,15 +5624,6 @@
       <c r="I19" s="1">
         <v>-123</v>
       </c>
-      <c r="J19" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K19" s="1">
-        <v>19</v>
-      </c>
-      <c r="L19" s="1">
-        <v>53</v>
-      </c>
       <c r="M19" s="1">
         <v>28</v>
       </c>
@@ -5803,17 +5859,11 @@
       <c r="I21" s="1">
         <v>-123</v>
       </c>
-      <c r="J21" s="1" t="s">
-        <v>62</v>
-      </c>
       <c r="K21" s="1">
         <v>42</v>
       </c>
       <c r="L21" s="1">
         <v>48</v>
-      </c>
-      <c r="M21" s="1">
-        <v>10</v>
       </c>
       <c r="N21" s="1">
         <v>1.1000000000000001</v>
@@ -6175,11 +6225,8 @@
       <c r="K24" s="1">
         <v>44</v>
       </c>
-      <c r="L24" s="1">
-        <v>42</v>
-      </c>
       <c r="M24" s="1">
-        <v>14</v>
+        <v>400</v>
       </c>
       <c r="N24" s="1">
         <v>1.18</v>
@@ -16178,7 +16225,7 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>469</v>
+        <v>137</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>13</v>
@@ -16262,7 +16309,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>470</v>
+        <v>146</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>172</v>
@@ -16481,7 +16528,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="12.711"/>
@@ -16517,16 +16564,58 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Texture fractions must be between 0 and 100.
+Affected samples:
+"22-OSN03-01" and "22-XTO07-03"</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Texture fractions must sum to 100 (+/- 1).
+Affected samples:
+"22-OSN03-01" and "22-UGU06-02"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>warning</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Invalid measurement_group values: "a" and "f".
-Valid options for English:
-"Physical", "Biological", "Chemical", "Plant Essential Macro Nutrients", and "Plant Essential Micro Nutrients"</t>
+          <t>At least two texture fractions must be provided to classify texture class.
+Affected samples:
+"22-OWZ06-02"</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>warning</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>One texture fraction is missing and will be computed as 100 minus the other two.
+Affected samples:
+"22-YIC08-01", "22-YGV09-02", and "22-XTO07-03"</t>
         </is>
       </c>
     </row>

</xml_diff>